<commit_message>
Update Marcela page (auto, 2026-06-02)
</commit_message>
<xml_diff>
--- a/public/marcela/Marcela_Loan_Tracker.xlsx
+++ b/public/marcela/Marcela_Loan_Tracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="66">
   <si>
     <t xml:space="preserve">Marcela Pool Loan Tracker</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t xml:space="preserve">Current Principal Balance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accrued Interest Receivable (Forborne)</t>
   </si>
   <si>
     <t xml:space="preserve">Total Outstanding</t>
@@ -1178,30 +1175,25 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E13" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <f aca="false">ROUND(C6*C7*(DATE(2025,9,1)-C9)/365,2)</f>
-        <v>945.21</v>
-      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
       <c r="E14" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F14" s="12" t="n">
-        <f aca="false">F12+F13</f>
-        <v>46384.42</v>
+        <f aca="false">F12</f>
+        <v>45439.21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="15"/>
       <c r="E15" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">IF(F12&lt;=0,0,IF(F7&lt;=0,F12,-PMT(C7/12,F7,F12)))</f>
@@ -1213,7 +1205,7 @@
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
       <c r="E16" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">IF(F6=0,0,F12-INDEX('Expected Schedule'!G6:G89,MIN(F6,84)))</f>
@@ -1229,7 +1221,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -1238,7 +1230,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
@@ -1268,7 +1260,7 @@
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -1277,7 +1269,7 @@
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C24" s="18"/>
       <c r="D24" s="18"/>
@@ -1286,7 +1278,7 @@
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C25" s="18"/>
       <c r="D25" s="18"/>
@@ -1295,7 +1287,7 @@
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C26" s="18"/>
       <c r="D26" s="18"/>
@@ -1304,7 +1296,7 @@
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C27" s="18"/>
       <c r="D27" s="18"/>
@@ -1313,7 +1305,7 @@
     </row>
     <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C28" s="18"/>
       <c r="D28" s="18"/>
@@ -1435,7 +1427,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
@@ -1447,7 +1439,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -1459,28 +1451,28 @@
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="F5" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="H5" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="I5" s="20" t="s">
         <v>38</v>
-      </c>
-      <c r="I5" s="20" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1492,7 +1484,7 @@
       </c>
       <c r="D6" s="21"/>
       <c r="E6" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
@@ -1501,7 +1493,7 @@
         <v>50000</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1516,7 +1508,7 @@
         <v>706.7</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F7" s="28" t="n">
         <f aca="false">IF(C7="","",ROUND(H6*Dashboard!$C$7/12,2))</f>
@@ -1531,7 +1523,7 @@
         <v>49501.63</v>
       </c>
       <c r="I7" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1546,7 +1538,7 @@
         <v>706.7</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">IF(C8="","",ROUND(H7*Dashboard!$C$7/12,2))</f>
@@ -1561,7 +1553,7 @@
         <v>49001.19</v>
       </c>
       <c r="I8" s="31" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1576,7 +1568,7 @@
         <v>706.7</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">IF(C9="","",ROUND(H8*Dashboard!$C$7/12,2))</f>
@@ -1591,7 +1583,7 @@
         <v>48498.66</v>
       </c>
       <c r="I9" s="31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1606,7 +1598,7 @@
         <v>706.7</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F10" s="28" t="n">
         <f aca="false">IF(C10="","",ROUND(H9*Dashboard!$C$7/12,2))</f>
@@ -1621,7 +1613,7 @@
         <v>47994.04</v>
       </c>
       <c r="I10" s="31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1636,7 +1628,7 @@
         <v>706.7</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F11" s="28" t="n">
         <f aca="false">IF(C11="","",ROUND(H10*Dashboard!$C$7/12,2))</f>
@@ -1651,7 +1643,7 @@
         <v>47487.32</v>
       </c>
       <c r="I11" s="31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1666,7 +1658,7 @@
         <v>706.7</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F12" s="28" t="n">
         <f aca="false">IF(C12="","",ROUND(H11*Dashboard!$C$7/12,2))</f>
@@ -1681,7 +1673,7 @@
         <v>46978.48</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1696,7 +1688,7 @@
         <v>706.7</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F13" s="28" t="n">
         <f aca="false">IF(C13="","",ROUND(H12*Dashboard!$C$7/12,2))</f>
@@ -1711,7 +1703,7 @@
         <v>46467.52</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1726,7 +1718,7 @@
         <v>706.7</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F14" s="28" t="n">
         <f aca="false">IF(C14="","",ROUND(H13*Dashboard!$C$7/12,2))</f>
@@ -1741,7 +1733,7 @@
         <v>45954.43</v>
       </c>
       <c r="I14" s="31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1756,7 +1748,7 @@
         <v>706.7</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F15" s="28" t="n">
         <f aca="false">IF(C15="","",ROUND(H14*Dashboard!$C$7/12,2))</f>
@@ -1771,7 +1763,7 @@
         <v>45439.21</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3612,7 +3604,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
@@ -3622,7 +3614,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -3632,22 +3624,22 @@
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="33" t="s">
-        <v>33</v>
-      </c>
       <c r="D5" s="33" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="33" t="s">
+      <c r="G5" s="33" t="s">
         <v>37</v>
-      </c>
-      <c r="G5" s="33" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5365,7 +5357,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C2" s="37"/>
       <c r="D2" s="37"/>
@@ -5374,7 +5366,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C3" s="38"/>
       <c r="D3" s="38"/>
@@ -5383,7 +5375,7 @@
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5" s="39"/>
       <c r="D5" s="39"/>
@@ -5401,7 +5393,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C7" s="41" t="n">
         <f aca="false">INDEX('Payment Register'!C7:C200,1)</f>
@@ -5410,31 +5402,31 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C8" s="42" t="n">
         <f aca="false">ROUND(Dashboard!C6*Dashboard!C7*(DATE(2025,9,1)-Dashboard!C9)/365,2)</f>
         <v>945.21</v>
       </c>
       <c r="D8" s="43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C9" s="44" t="n">
         <f aca="false">-ROUND(Dashboard!C6*Dashboard!C7*(DATE(2025,9,1)-Dashboard!C9)/365,2)</f>
         <v>-945.21</v>
       </c>
       <c r="D9" s="45" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C10" s="42" t="n">
         <f aca="false">C8+C9</f>
@@ -5443,19 +5435,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="40" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C11" s="41" t="n">
         <f aca="false">DATE(2025,9,1)</f>
         <v>45901</v>
       </c>
       <c r="D11" s="46" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="47" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C13" s="47"/>
       <c r="D13" s="47"/>

</xml_diff>

<commit_message>
Update Marcela page (auto, 2026-06-26)
</commit_message>
<xml_diff>
--- a/public/marcela/Marcela_Loan_Tracker.xlsx
+++ b/public/marcela/Marcela_Loan_Tracker.xlsx
@@ -224,7 +224,7 @@
     <t xml:space="preserve">ANCHOR</t>
   </si>
   <si>
-    <t xml:space="preserve">Loan funded 4/16/25. From funding through Sept 1, 2025, interest accrued at 5% APR (day-count) totaling $945.21. The lender is currently forbearing collection of this amount; it is held in reserve as accrued interest receivable and may be added back to the outstanding balance if the loan is called or otherwise accelerated. From the Effective Loan Start of 9/1/25 forward, interest accrues on a monthly cycle: each cycle charges one month of interest at 5%/12 = 0.4167% on the prior balance. Expected payments are due on the 5th of each month. Payments made within the same monthly cycle do not change the interest charged for that cycle.</t>
+    <t xml:space="preserve">Loan funded 4/16/2025. Borrower's first payment was received 10/1/2025. Across the 168-day interval from funding to first payment, interest accrued at 5% APR (actual/365 day count) totaling $1,150.68. The lender is currently forbearing collection of this pre-payment interest and has booked it in reserve. It is not included in the borrower-facing Total Outstanding on the Dashboard and is not reflected in the public statement page. The lender reserves the right to recall this forborne interest in the event of acceleration, default, prepayment, or material change of circumstances. The monthly accrual cycle on the Payment Register begins 10/1/2025 with a clean balance of $50,000.</t>
   </si>
 </sst>
 </file>
@@ -1125,8 +1125,8 @@
         <v>11</v>
       </c>
       <c r="F9" s="12" t="n">
-        <f aca="false">ROUND(C6*C7*(DATE(2025,9,1)-C9)/365,2)+SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!F7:F200)</f>
-        <v>2744.72</v>
+        <f aca="false">ROUND(C6*C7*(DATE(2025,10,1)-C9)/365,2)+SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!F7:F200)</f>
+        <v>2950.19</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1134,7 +1134,7 @@
         <v>12</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>45809</v>
+        <v>45931</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>13</v>
@@ -5405,8 +5405,8 @@
         <v>58</v>
       </c>
       <c r="C8" s="42" t="n">
-        <f aca="false">ROUND(Dashboard!C6*Dashboard!C7*(DATE(2025,9,1)-Dashboard!C9)/365,2)</f>
-        <v>945.21</v>
+        <f aca="false">ROUND(Dashboard!C6*Dashboard!C7*(DATE(2025,10,1)-Dashboard!C9)/365,2)</f>
+        <v>1150.68</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>59</v>
@@ -5417,8 +5417,8 @@
         <v>60</v>
       </c>
       <c r="C9" s="44" t="n">
-        <f aca="false">-ROUND(Dashboard!C6*Dashboard!C7*(DATE(2025,9,1)-Dashboard!C9)/365,2)</f>
-        <v>-945.21</v>
+        <f aca="false">-ROUND(Dashboard!C6*Dashboard!C7*(DATE(2025,10,1)-Dashboard!C9)/365,2)</f>
+        <v>-1150.68</v>
       </c>
       <c r="D9" s="45" t="s">
         <v>61</v>
@@ -5438,8 +5438,8 @@
         <v>63</v>
       </c>
       <c r="C11" s="41" t="n">
-        <f aca="false">DATE(2025,9,1)</f>
-        <v>45901</v>
+        <f aca="false">DATE(2025,10,1)</f>
+        <v>45931</v>
       </c>
       <c r="D11" s="46" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Update Marcela page (auto, 2026-07-14): payment #14 6/29/2026, balance $42,830.71
</commit_message>
<xml_diff>
--- a/public/marcela/Marcela_Loan_Tracker.xlsx
+++ b/public/marcela/Marcela_Loan_Tracker.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="58">
   <si>
     <t xml:space="preserve">Marcela Pool Loan Tracker</t>
   </si>
@@ -188,6 +188,9 @@
   </si>
   <si>
     <t xml:space="preserve">BofA. Memo 'Loan payment'. Conf# 0K6GDYWCK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-imported. Conf# 0K788773T. Memo: Pool loan payment July 1 2026 (paid early 6/29)</t>
   </si>
   <si>
     <t xml:space="preserve">Expected Payment Schedule (84 Months, Payments Due 5th of Month)</t>
@@ -539,12 +542,12 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -732,34 +735,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -957,7 +960,7 @@
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">COUNT('Payment Register'!C7:C200)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -972,7 +975,7 @@
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">C8-F6</f>
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -987,7 +990,7 @@
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!D7:D200)</f>
-        <v>9187.1</v>
+        <v>9893.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1002,7 +1005,7 @@
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!F7:F200)</f>
-        <v>2543.86</v>
+        <v>2724.51</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1017,7 +1020,7 @@
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!F7:F200)</f>
-        <v>2543.86</v>
+        <v>2724.51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1032,7 +1035,7 @@
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">SUMIF('Payment Register'!C7:C200,"&gt;0",'Payment Register'!G7:G200)</f>
-        <v>6643.24</v>
+        <v>7169.29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1047,7 +1050,7 @@
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">LOOKUP(2,1/('Payment Register'!H6:H200&lt;&gt;""),'Payment Register'!H6:H200)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1068,7 +1071,7 @@
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">IF(F12&lt;=0,0,IF(F7&lt;=0,F12,-PMT(C7/12,F7,F12)))</f>
-        <v>706.694406014719</v>
+        <v>706.694261466509</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1758,33 +1761,41 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="28" t="str">
+      <c r="B20" s="28" t="n">
         <f aca="false">IF(C20="","",MAX($B$6:B19)+1)</f>
-        <v/>
-      </c>
-      <c r="C20" s="34"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="30" t="str">
+        <v>14</v>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>46202</v>
+      </c>
+      <c r="D20" s="30" t="n">
+        <v>706.7</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="30" t="n">
         <f aca="false">IF(C20="","",ROUND(H19*Dashboard!$C$7/12,2))</f>
-        <v/>
-      </c>
-      <c r="G20" s="30" t="str">
+        <v>180.65</v>
+      </c>
+      <c r="G20" s="30" t="n">
         <f aca="false">IF(C20="","",IF(OR(D20="",ISBLANK(D20)),-F20,D20-F20))</f>
-        <v/>
+        <v>526.05</v>
       </c>
       <c r="H20" s="32" t="n">
         <f aca="false">IF(C20="",H19,H19-G20)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I20" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I20" s="34" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="28" t="str">
         <f aca="false">IF(C21="","",MAX($B$6:B20)+1)</f>
         <v/>
       </c>
-      <c r="C21" s="34"/>
+      <c r="C21" s="35"/>
       <c r="D21" s="30"/>
       <c r="E21" s="31"/>
       <c r="F21" s="30" t="str">
@@ -1797,16 +1808,16 @@
       </c>
       <c r="H21" s="32" t="n">
         <f aca="false">IF(C21="",H20,H20-G21)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I21" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="28" t="str">
         <f aca="false">IF(C22="","",MAX($B$6:B21)+1)</f>
         <v/>
       </c>
-      <c r="C22" s="34"/>
+      <c r="C22" s="35"/>
       <c r="D22" s="30"/>
       <c r="E22" s="31"/>
       <c r="F22" s="30" t="str">
@@ -1819,16 +1830,16 @@
       </c>
       <c r="H22" s="32" t="n">
         <f aca="false">IF(C22="",H21,H21-G22)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I22" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I22" s="34"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="28" t="str">
         <f aca="false">IF(C23="","",MAX($B$6:B22)+1)</f>
         <v/>
       </c>
-      <c r="C23" s="34"/>
+      <c r="C23" s="35"/>
       <c r="D23" s="30"/>
       <c r="E23" s="31"/>
       <c r="F23" s="30" t="str">
@@ -1841,16 +1852,16 @@
       </c>
       <c r="H23" s="32" t="n">
         <f aca="false">IF(C23="",H22,H22-G23)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I23" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="28" t="str">
         <f aca="false">IF(C24="","",MAX($B$6:B23)+1)</f>
         <v/>
       </c>
-      <c r="C24" s="34"/>
+      <c r="C24" s="35"/>
       <c r="D24" s="30"/>
       <c r="E24" s="31"/>
       <c r="F24" s="30" t="str">
@@ -1863,16 +1874,16 @@
       </c>
       <c r="H24" s="32" t="n">
         <f aca="false">IF(C24="",H23,H23-G24)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I24" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I24" s="34"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="28" t="str">
         <f aca="false">IF(C25="","",MAX($B$6:B24)+1)</f>
         <v/>
       </c>
-      <c r="C25" s="34"/>
+      <c r="C25" s="35"/>
       <c r="D25" s="30"/>
       <c r="E25" s="31"/>
       <c r="F25" s="30" t="str">
@@ -1885,16 +1896,16 @@
       </c>
       <c r="H25" s="32" t="n">
         <f aca="false">IF(C25="",H24,H24-G25)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I25" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="28" t="str">
         <f aca="false">IF(C26="","",MAX($B$6:B25)+1)</f>
         <v/>
       </c>
-      <c r="C26" s="34"/>
+      <c r="C26" s="35"/>
       <c r="D26" s="30"/>
       <c r="E26" s="31"/>
       <c r="F26" s="30" t="str">
@@ -1907,16 +1918,16 @@
       </c>
       <c r="H26" s="32" t="n">
         <f aca="false">IF(C26="",H25,H25-G26)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I26" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I26" s="34"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="28" t="str">
         <f aca="false">IF(C27="","",MAX($B$6:B26)+1)</f>
         <v/>
       </c>
-      <c r="C27" s="34"/>
+      <c r="C27" s="35"/>
       <c r="D27" s="30"/>
       <c r="E27" s="31"/>
       <c r="F27" s="30" t="str">
@@ -1929,16 +1940,16 @@
       </c>
       <c r="H27" s="32" t="n">
         <f aca="false">IF(C27="",H26,H26-G27)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I27" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="28" t="str">
         <f aca="false">IF(C28="","",MAX($B$6:B27)+1)</f>
         <v/>
       </c>
-      <c r="C28" s="34"/>
+      <c r="C28" s="35"/>
       <c r="D28" s="30"/>
       <c r="E28" s="31"/>
       <c r="F28" s="30" t="str">
@@ -1951,16 +1962,16 @@
       </c>
       <c r="H28" s="32" t="n">
         <f aca="false">IF(C28="",H27,H27-G28)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I28" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I28" s="34"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="28" t="str">
         <f aca="false">IF(C29="","",MAX($B$6:B28)+1)</f>
         <v/>
       </c>
-      <c r="C29" s="34"/>
+      <c r="C29" s="35"/>
       <c r="D29" s="30"/>
       <c r="E29" s="31"/>
       <c r="F29" s="30" t="str">
@@ -1973,16 +1984,16 @@
       </c>
       <c r="H29" s="32" t="n">
         <f aca="false">IF(C29="",H28,H28-G29)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I29" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="28" t="str">
         <f aca="false">IF(C30="","",MAX($B$6:B29)+1)</f>
         <v/>
       </c>
-      <c r="C30" s="34"/>
+      <c r="C30" s="35"/>
       <c r="D30" s="30"/>
       <c r="E30" s="31"/>
       <c r="F30" s="30" t="str">
@@ -1995,16 +2006,16 @@
       </c>
       <c r="H30" s="32" t="n">
         <f aca="false">IF(C30="",H29,H29-G30)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I30" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I30" s="34"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="28" t="str">
         <f aca="false">IF(C31="","",MAX($B$6:B30)+1)</f>
         <v/>
       </c>
-      <c r="C31" s="34"/>
+      <c r="C31" s="35"/>
       <c r="D31" s="30"/>
       <c r="E31" s="31"/>
       <c r="F31" s="30" t="str">
@@ -2017,16 +2028,16 @@
       </c>
       <c r="H31" s="32" t="n">
         <f aca="false">IF(C31="",H30,H30-G31)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I31" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="28" t="str">
         <f aca="false">IF(C32="","",MAX($B$6:B31)+1)</f>
         <v/>
       </c>
-      <c r="C32" s="34"/>
+      <c r="C32" s="35"/>
       <c r="D32" s="30"/>
       <c r="E32" s="31"/>
       <c r="F32" s="30" t="str">
@@ -2039,16 +2050,16 @@
       </c>
       <c r="H32" s="32" t="n">
         <f aca="false">IF(C32="",H31,H31-G32)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I32" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I32" s="34"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="28" t="str">
         <f aca="false">IF(C33="","",MAX($B$6:B32)+1)</f>
         <v/>
       </c>
-      <c r="C33" s="34"/>
+      <c r="C33" s="35"/>
       <c r="D33" s="30"/>
       <c r="E33" s="31"/>
       <c r="F33" s="30" t="str">
@@ -2061,16 +2072,16 @@
       </c>
       <c r="H33" s="32" t="n">
         <f aca="false">IF(C33="",H32,H32-G33)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I33" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I33" s="34"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="28" t="str">
         <f aca="false">IF(C34="","",MAX($B$6:B33)+1)</f>
         <v/>
       </c>
-      <c r="C34" s="34"/>
+      <c r="C34" s="35"/>
       <c r="D34" s="30"/>
       <c r="E34" s="31"/>
       <c r="F34" s="30" t="str">
@@ -2083,16 +2094,16 @@
       </c>
       <c r="H34" s="32" t="n">
         <f aca="false">IF(C34="",H33,H33-G34)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I34" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I34" s="34"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="28" t="str">
         <f aca="false">IF(C35="","",MAX($B$6:B34)+1)</f>
         <v/>
       </c>
-      <c r="C35" s="34"/>
+      <c r="C35" s="35"/>
       <c r="D35" s="30"/>
       <c r="E35" s="31"/>
       <c r="F35" s="30" t="str">
@@ -2105,16 +2116,16 @@
       </c>
       <c r="H35" s="32" t="n">
         <f aca="false">IF(C35="",H34,H34-G35)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I35" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I35" s="34"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="28" t="str">
         <f aca="false">IF(C36="","",MAX($B$6:B35)+1)</f>
         <v/>
       </c>
-      <c r="C36" s="34"/>
+      <c r="C36" s="35"/>
       <c r="D36" s="30"/>
       <c r="E36" s="31"/>
       <c r="F36" s="30" t="str">
@@ -2127,16 +2138,16 @@
       </c>
       <c r="H36" s="32" t="n">
         <f aca="false">IF(C36="",H35,H35-G36)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I36" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I36" s="34"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="28" t="str">
         <f aca="false">IF(C37="","",MAX($B$6:B36)+1)</f>
         <v/>
       </c>
-      <c r="C37" s="34"/>
+      <c r="C37" s="35"/>
       <c r="D37" s="30"/>
       <c r="E37" s="31"/>
       <c r="F37" s="30" t="str">
@@ -2149,16 +2160,16 @@
       </c>
       <c r="H37" s="32" t="n">
         <f aca="false">IF(C37="",H36,H36-G37)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I37" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I37" s="34"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="28" t="str">
         <f aca="false">IF(C38="","",MAX($B$6:B37)+1)</f>
         <v/>
       </c>
-      <c r="C38" s="34"/>
+      <c r="C38" s="35"/>
       <c r="D38" s="30"/>
       <c r="E38" s="31"/>
       <c r="F38" s="30" t="str">
@@ -2171,16 +2182,16 @@
       </c>
       <c r="H38" s="32" t="n">
         <f aca="false">IF(C38="",H37,H37-G38)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I38" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I38" s="34"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="28" t="str">
         <f aca="false">IF(C39="","",MAX($B$6:B38)+1)</f>
         <v/>
       </c>
-      <c r="C39" s="34"/>
+      <c r="C39" s="35"/>
       <c r="D39" s="30"/>
       <c r="E39" s="31"/>
       <c r="F39" s="30" t="str">
@@ -2193,16 +2204,16 @@
       </c>
       <c r="H39" s="32" t="n">
         <f aca="false">IF(C39="",H38,H38-G39)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I39" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I39" s="34"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="28" t="str">
         <f aca="false">IF(C40="","",MAX($B$6:B39)+1)</f>
         <v/>
       </c>
-      <c r="C40" s="34"/>
+      <c r="C40" s="35"/>
       <c r="D40" s="30"/>
       <c r="E40" s="31"/>
       <c r="F40" s="30" t="str">
@@ -2215,16 +2226,16 @@
       </c>
       <c r="H40" s="32" t="n">
         <f aca="false">IF(C40="",H39,H39-G40)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I40" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I40" s="34"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="28" t="str">
         <f aca="false">IF(C41="","",MAX($B$6:B40)+1)</f>
         <v/>
       </c>
-      <c r="C41" s="34"/>
+      <c r="C41" s="35"/>
       <c r="D41" s="30"/>
       <c r="E41" s="31"/>
       <c r="F41" s="30" t="str">
@@ -2237,16 +2248,16 @@
       </c>
       <c r="H41" s="32" t="n">
         <f aca="false">IF(C41="",H40,H40-G41)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I41" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I41" s="34"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="28" t="str">
         <f aca="false">IF(C42="","",MAX($B$6:B41)+1)</f>
         <v/>
       </c>
-      <c r="C42" s="34"/>
+      <c r="C42" s="35"/>
       <c r="D42" s="30"/>
       <c r="E42" s="31"/>
       <c r="F42" s="30" t="str">
@@ -2259,16 +2270,16 @@
       </c>
       <c r="H42" s="32" t="n">
         <f aca="false">IF(C42="",H41,H41-G42)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I42" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I42" s="34"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="28" t="str">
         <f aca="false">IF(C43="","",MAX($B$6:B42)+1)</f>
         <v/>
       </c>
-      <c r="C43" s="34"/>
+      <c r="C43" s="35"/>
       <c r="D43" s="30"/>
       <c r="E43" s="31"/>
       <c r="F43" s="30" t="str">
@@ -2281,16 +2292,16 @@
       </c>
       <c r="H43" s="32" t="n">
         <f aca="false">IF(C43="",H42,H42-G43)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I43" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I43" s="34"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="28" t="str">
         <f aca="false">IF(C44="","",MAX($B$6:B43)+1)</f>
         <v/>
       </c>
-      <c r="C44" s="34"/>
+      <c r="C44" s="35"/>
       <c r="D44" s="30"/>
       <c r="E44" s="31"/>
       <c r="F44" s="30" t="str">
@@ -2303,16 +2314,16 @@
       </c>
       <c r="H44" s="32" t="n">
         <f aca="false">IF(C44="",H43,H43-G44)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I44" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I44" s="34"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="28" t="str">
         <f aca="false">IF(C45="","",MAX($B$6:B44)+1)</f>
         <v/>
       </c>
-      <c r="C45" s="34"/>
+      <c r="C45" s="35"/>
       <c r="D45" s="30"/>
       <c r="E45" s="31"/>
       <c r="F45" s="30" t="str">
@@ -2325,16 +2336,16 @@
       </c>
       <c r="H45" s="32" t="n">
         <f aca="false">IF(C45="",H44,H44-G45)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I45" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I45" s="34"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="28" t="str">
         <f aca="false">IF(C46="","",MAX($B$6:B45)+1)</f>
         <v/>
       </c>
-      <c r="C46" s="34"/>
+      <c r="C46" s="35"/>
       <c r="D46" s="30"/>
       <c r="E46" s="31"/>
       <c r="F46" s="30" t="str">
@@ -2347,16 +2358,16 @@
       </c>
       <c r="H46" s="32" t="n">
         <f aca="false">IF(C46="",H45,H45-G46)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I46" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I46" s="34"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="28" t="str">
         <f aca="false">IF(C47="","",MAX($B$6:B46)+1)</f>
         <v/>
       </c>
-      <c r="C47" s="34"/>
+      <c r="C47" s="35"/>
       <c r="D47" s="30"/>
       <c r="E47" s="31"/>
       <c r="F47" s="30" t="str">
@@ -2369,16 +2380,16 @@
       </c>
       <c r="H47" s="32" t="n">
         <f aca="false">IF(C47="",H46,H46-G47)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I47" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I47" s="34"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="28" t="str">
         <f aca="false">IF(C48="","",MAX($B$6:B47)+1)</f>
         <v/>
       </c>
-      <c r="C48" s="34"/>
+      <c r="C48" s="35"/>
       <c r="D48" s="30"/>
       <c r="E48" s="31"/>
       <c r="F48" s="30" t="str">
@@ -2391,16 +2402,16 @@
       </c>
       <c r="H48" s="32" t="n">
         <f aca="false">IF(C48="",H47,H47-G48)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I48" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I48" s="34"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="28" t="str">
         <f aca="false">IF(C49="","",MAX($B$6:B48)+1)</f>
         <v/>
       </c>
-      <c r="C49" s="34"/>
+      <c r="C49" s="35"/>
       <c r="D49" s="30"/>
       <c r="E49" s="31"/>
       <c r="F49" s="30" t="str">
@@ -2413,16 +2424,16 @@
       </c>
       <c r="H49" s="32" t="n">
         <f aca="false">IF(C49="",H48,H48-G49)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I49" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I49" s="34"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="28" t="str">
         <f aca="false">IF(C50="","",MAX($B$6:B49)+1)</f>
         <v/>
       </c>
-      <c r="C50" s="34"/>
+      <c r="C50" s="35"/>
       <c r="D50" s="30"/>
       <c r="E50" s="31"/>
       <c r="F50" s="30" t="str">
@@ -2435,16 +2446,16 @@
       </c>
       <c r="H50" s="32" t="n">
         <f aca="false">IF(C50="",H49,H49-G50)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I50" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I50" s="34"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="28" t="str">
         <f aca="false">IF(C51="","",MAX($B$6:B50)+1)</f>
         <v/>
       </c>
-      <c r="C51" s="34"/>
+      <c r="C51" s="35"/>
       <c r="D51" s="30"/>
       <c r="E51" s="31"/>
       <c r="F51" s="30" t="str">
@@ -2457,16 +2468,16 @@
       </c>
       <c r="H51" s="32" t="n">
         <f aca="false">IF(C51="",H50,H50-G51)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I51" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I51" s="34"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="28" t="str">
         <f aca="false">IF(C52="","",MAX($B$6:B51)+1)</f>
         <v/>
       </c>
-      <c r="C52" s="34"/>
+      <c r="C52" s="35"/>
       <c r="D52" s="30"/>
       <c r="E52" s="31"/>
       <c r="F52" s="30" t="str">
@@ -2479,16 +2490,16 @@
       </c>
       <c r="H52" s="32" t="n">
         <f aca="false">IF(C52="",H51,H51-G52)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I52" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I52" s="34"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="28" t="str">
         <f aca="false">IF(C53="","",MAX($B$6:B52)+1)</f>
         <v/>
       </c>
-      <c r="C53" s="34"/>
+      <c r="C53" s="35"/>
       <c r="D53" s="30"/>
       <c r="E53" s="31"/>
       <c r="F53" s="30" t="str">
@@ -2501,16 +2512,16 @@
       </c>
       <c r="H53" s="32" t="n">
         <f aca="false">IF(C53="",H52,H52-G53)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I53" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I53" s="34"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="28" t="str">
         <f aca="false">IF(C54="","",MAX($B$6:B53)+1)</f>
         <v/>
       </c>
-      <c r="C54" s="34"/>
+      <c r="C54" s="35"/>
       <c r="D54" s="30"/>
       <c r="E54" s="31"/>
       <c r="F54" s="30" t="str">
@@ -2523,16 +2534,16 @@
       </c>
       <c r="H54" s="32" t="n">
         <f aca="false">IF(C54="",H53,H53-G54)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I54" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I54" s="34"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="28" t="str">
         <f aca="false">IF(C55="","",MAX($B$6:B54)+1)</f>
         <v/>
       </c>
-      <c r="C55" s="34"/>
+      <c r="C55" s="35"/>
       <c r="D55" s="30"/>
       <c r="E55" s="31"/>
       <c r="F55" s="30" t="str">
@@ -2545,16 +2556,16 @@
       </c>
       <c r="H55" s="32" t="n">
         <f aca="false">IF(C55="",H54,H54-G55)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I55" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I55" s="34"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="28" t="str">
         <f aca="false">IF(C56="","",MAX($B$6:B55)+1)</f>
         <v/>
       </c>
-      <c r="C56" s="34"/>
+      <c r="C56" s="35"/>
       <c r="D56" s="30"/>
       <c r="E56" s="31"/>
       <c r="F56" s="30" t="str">
@@ -2567,16 +2578,16 @@
       </c>
       <c r="H56" s="32" t="n">
         <f aca="false">IF(C56="",H55,H55-G56)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I56" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I56" s="34"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="28" t="str">
         <f aca="false">IF(C57="","",MAX($B$6:B56)+1)</f>
         <v/>
       </c>
-      <c r="C57" s="34"/>
+      <c r="C57" s="35"/>
       <c r="D57" s="30"/>
       <c r="E57" s="31"/>
       <c r="F57" s="30" t="str">
@@ -2589,16 +2600,16 @@
       </c>
       <c r="H57" s="32" t="n">
         <f aca="false">IF(C57="",H56,H56-G57)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I57" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I57" s="34"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="28" t="str">
         <f aca="false">IF(C58="","",MAX($B$6:B57)+1)</f>
         <v/>
       </c>
-      <c r="C58" s="34"/>
+      <c r="C58" s="35"/>
       <c r="D58" s="30"/>
       <c r="E58" s="31"/>
       <c r="F58" s="30" t="str">
@@ -2611,16 +2622,16 @@
       </c>
       <c r="H58" s="32" t="n">
         <f aca="false">IF(C58="",H57,H57-G58)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I58" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I58" s="34"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="28" t="str">
         <f aca="false">IF(C59="","",MAX($B$6:B58)+1)</f>
         <v/>
       </c>
-      <c r="C59" s="34"/>
+      <c r="C59" s="35"/>
       <c r="D59" s="30"/>
       <c r="E59" s="31"/>
       <c r="F59" s="30" t="str">
@@ -2633,16 +2644,16 @@
       </c>
       <c r="H59" s="32" t="n">
         <f aca="false">IF(C59="",H58,H58-G59)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I59" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I59" s="34"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="28" t="str">
         <f aca="false">IF(C60="","",MAX($B$6:B59)+1)</f>
         <v/>
       </c>
-      <c r="C60" s="34"/>
+      <c r="C60" s="35"/>
       <c r="D60" s="30"/>
       <c r="E60" s="31"/>
       <c r="F60" s="30" t="str">
@@ -2655,16 +2666,16 @@
       </c>
       <c r="H60" s="32" t="n">
         <f aca="false">IF(C60="",H59,H59-G60)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I60" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I60" s="34"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="28" t="str">
         <f aca="false">IF(C61="","",MAX($B$6:B60)+1)</f>
         <v/>
       </c>
-      <c r="C61" s="34"/>
+      <c r="C61" s="35"/>
       <c r="D61" s="30"/>
       <c r="E61" s="31"/>
       <c r="F61" s="30" t="str">
@@ -2677,16 +2688,16 @@
       </c>
       <c r="H61" s="32" t="n">
         <f aca="false">IF(C61="",H60,H60-G61)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I61" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I61" s="34"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="28" t="str">
         <f aca="false">IF(C62="","",MAX($B$6:B61)+1)</f>
         <v/>
       </c>
-      <c r="C62" s="34"/>
+      <c r="C62" s="35"/>
       <c r="D62" s="30"/>
       <c r="E62" s="31"/>
       <c r="F62" s="30" t="str">
@@ -2699,16 +2710,16 @@
       </c>
       <c r="H62" s="32" t="n">
         <f aca="false">IF(C62="",H61,H61-G62)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I62" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I62" s="34"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="28" t="str">
         <f aca="false">IF(C63="","",MAX($B$6:B62)+1)</f>
         <v/>
       </c>
-      <c r="C63" s="34"/>
+      <c r="C63" s="35"/>
       <c r="D63" s="30"/>
       <c r="E63" s="31"/>
       <c r="F63" s="30" t="str">
@@ -2721,16 +2732,16 @@
       </c>
       <c r="H63" s="32" t="n">
         <f aca="false">IF(C63="",H62,H62-G63)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I63" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I63" s="34"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="28" t="str">
         <f aca="false">IF(C64="","",MAX($B$6:B63)+1)</f>
         <v/>
       </c>
-      <c r="C64" s="34"/>
+      <c r="C64" s="35"/>
       <c r="D64" s="30"/>
       <c r="E64" s="31"/>
       <c r="F64" s="30" t="str">
@@ -2743,16 +2754,16 @@
       </c>
       <c r="H64" s="32" t="n">
         <f aca="false">IF(C64="",H63,H63-G64)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I64" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I64" s="34"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="28" t="str">
         <f aca="false">IF(C65="","",MAX($B$6:B64)+1)</f>
         <v/>
       </c>
-      <c r="C65" s="34"/>
+      <c r="C65" s="35"/>
       <c r="D65" s="30"/>
       <c r="E65" s="31"/>
       <c r="F65" s="30" t="str">
@@ -2765,16 +2776,16 @@
       </c>
       <c r="H65" s="32" t="n">
         <f aca="false">IF(C65="",H64,H64-G65)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I65" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I65" s="34"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="28" t="str">
         <f aca="false">IF(C66="","",MAX($B$6:B65)+1)</f>
         <v/>
       </c>
-      <c r="C66" s="34"/>
+      <c r="C66" s="35"/>
       <c r="D66" s="30"/>
       <c r="E66" s="31"/>
       <c r="F66" s="30" t="str">
@@ -2787,16 +2798,16 @@
       </c>
       <c r="H66" s="32" t="n">
         <f aca="false">IF(C66="",H65,H65-G66)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I66" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I66" s="34"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="28" t="str">
         <f aca="false">IF(C67="","",MAX($B$6:B66)+1)</f>
         <v/>
       </c>
-      <c r="C67" s="34"/>
+      <c r="C67" s="35"/>
       <c r="D67" s="30"/>
       <c r="E67" s="31"/>
       <c r="F67" s="30" t="str">
@@ -2809,16 +2820,16 @@
       </c>
       <c r="H67" s="32" t="n">
         <f aca="false">IF(C67="",H66,H66-G67)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I67" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I67" s="34"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="28" t="str">
         <f aca="false">IF(C68="","",MAX($B$6:B67)+1)</f>
         <v/>
       </c>
-      <c r="C68" s="34"/>
+      <c r="C68" s="35"/>
       <c r="D68" s="30"/>
       <c r="E68" s="31"/>
       <c r="F68" s="30" t="str">
@@ -2831,16 +2842,16 @@
       </c>
       <c r="H68" s="32" t="n">
         <f aca="false">IF(C68="",H67,H67-G68)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I68" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I68" s="34"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="28" t="str">
         <f aca="false">IF(C69="","",MAX($B$6:B68)+1)</f>
         <v/>
       </c>
-      <c r="C69" s="34"/>
+      <c r="C69" s="35"/>
       <c r="D69" s="30"/>
       <c r="E69" s="31"/>
       <c r="F69" s="30" t="str">
@@ -2853,16 +2864,16 @@
       </c>
       <c r="H69" s="32" t="n">
         <f aca="false">IF(C69="",H68,H68-G69)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I69" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I69" s="34"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="28" t="str">
         <f aca="false">IF(C70="","",MAX($B$6:B69)+1)</f>
         <v/>
       </c>
-      <c r="C70" s="34"/>
+      <c r="C70" s="35"/>
       <c r="D70" s="30"/>
       <c r="E70" s="31"/>
       <c r="F70" s="30" t="str">
@@ -2875,16 +2886,16 @@
       </c>
       <c r="H70" s="32" t="n">
         <f aca="false">IF(C70="",H69,H69-G70)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I70" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I70" s="34"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="28" t="str">
         <f aca="false">IF(C71="","",MAX($B$6:B70)+1)</f>
         <v/>
       </c>
-      <c r="C71" s="34"/>
+      <c r="C71" s="35"/>
       <c r="D71" s="30"/>
       <c r="E71" s="31"/>
       <c r="F71" s="30" t="str">
@@ -2897,16 +2908,16 @@
       </c>
       <c r="H71" s="32" t="n">
         <f aca="false">IF(C71="",H70,H70-G71)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I71" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I71" s="34"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="28" t="str">
         <f aca="false">IF(C72="","",MAX($B$6:B71)+1)</f>
         <v/>
       </c>
-      <c r="C72" s="34"/>
+      <c r="C72" s="35"/>
       <c r="D72" s="30"/>
       <c r="E72" s="31"/>
       <c r="F72" s="30" t="str">
@@ -2919,16 +2930,16 @@
       </c>
       <c r="H72" s="32" t="n">
         <f aca="false">IF(C72="",H71,H71-G72)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I72" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I72" s="34"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B73" s="28" t="str">
         <f aca="false">IF(C73="","",MAX($B$6:B72)+1)</f>
         <v/>
       </c>
-      <c r="C73" s="34"/>
+      <c r="C73" s="35"/>
       <c r="D73" s="30"/>
       <c r="E73" s="31"/>
       <c r="F73" s="30" t="str">
@@ -2941,16 +2952,16 @@
       </c>
       <c r="H73" s="32" t="n">
         <f aca="false">IF(C73="",H72,H72-G73)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I73" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I73" s="34"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="28" t="str">
         <f aca="false">IF(C74="","",MAX($B$6:B73)+1)</f>
         <v/>
       </c>
-      <c r="C74" s="34"/>
+      <c r="C74" s="35"/>
       <c r="D74" s="30"/>
       <c r="E74" s="31"/>
       <c r="F74" s="30" t="str">
@@ -2963,16 +2974,16 @@
       </c>
       <c r="H74" s="32" t="n">
         <f aca="false">IF(C74="",H73,H73-G74)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I74" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I74" s="34"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="28" t="str">
         <f aca="false">IF(C75="","",MAX($B$6:B74)+1)</f>
         <v/>
       </c>
-      <c r="C75" s="34"/>
+      <c r="C75" s="35"/>
       <c r="D75" s="30"/>
       <c r="E75" s="31"/>
       <c r="F75" s="30" t="str">
@@ -2985,16 +2996,16 @@
       </c>
       <c r="H75" s="32" t="n">
         <f aca="false">IF(C75="",H74,H74-G75)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I75" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I75" s="34"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="28" t="str">
         <f aca="false">IF(C76="","",MAX($B$6:B75)+1)</f>
         <v/>
       </c>
-      <c r="C76" s="34"/>
+      <c r="C76" s="35"/>
       <c r="D76" s="30"/>
       <c r="E76" s="31"/>
       <c r="F76" s="30" t="str">
@@ -3007,16 +3018,16 @@
       </c>
       <c r="H76" s="32" t="n">
         <f aca="false">IF(C76="",H75,H75-G76)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I76" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I76" s="34"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="28" t="str">
         <f aca="false">IF(C77="","",MAX($B$6:B76)+1)</f>
         <v/>
       </c>
-      <c r="C77" s="34"/>
+      <c r="C77" s="35"/>
       <c r="D77" s="30"/>
       <c r="E77" s="31"/>
       <c r="F77" s="30" t="str">
@@ -3029,16 +3040,16 @@
       </c>
       <c r="H77" s="32" t="n">
         <f aca="false">IF(C77="",H76,H76-G77)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I77" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I77" s="34"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="28" t="str">
         <f aca="false">IF(C78="","",MAX($B$6:B77)+1)</f>
         <v/>
       </c>
-      <c r="C78" s="34"/>
+      <c r="C78" s="35"/>
       <c r="D78" s="30"/>
       <c r="E78" s="31"/>
       <c r="F78" s="30" t="str">
@@ -3051,16 +3062,16 @@
       </c>
       <c r="H78" s="32" t="n">
         <f aca="false">IF(C78="",H77,H77-G78)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I78" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I78" s="34"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B79" s="28" t="str">
         <f aca="false">IF(C79="","",MAX($B$6:B78)+1)</f>
         <v/>
       </c>
-      <c r="C79" s="34"/>
+      <c r="C79" s="35"/>
       <c r="D79" s="30"/>
       <c r="E79" s="31"/>
       <c r="F79" s="30" t="str">
@@ -3073,16 +3084,16 @@
       </c>
       <c r="H79" s="32" t="n">
         <f aca="false">IF(C79="",H78,H78-G79)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I79" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I79" s="34"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="28" t="str">
         <f aca="false">IF(C80="","",MAX($B$6:B79)+1)</f>
         <v/>
       </c>
-      <c r="C80" s="34"/>
+      <c r="C80" s="35"/>
       <c r="D80" s="30"/>
       <c r="E80" s="31"/>
       <c r="F80" s="30" t="str">
@@ -3095,16 +3106,16 @@
       </c>
       <c r="H80" s="32" t="n">
         <f aca="false">IF(C80="",H79,H79-G80)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I80" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I80" s="34"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B81" s="28" t="str">
         <f aca="false">IF(C81="","",MAX($B$6:B80)+1)</f>
         <v/>
       </c>
-      <c r="C81" s="34"/>
+      <c r="C81" s="35"/>
       <c r="D81" s="30"/>
       <c r="E81" s="31"/>
       <c r="F81" s="30" t="str">
@@ -3117,16 +3128,16 @@
       </c>
       <c r="H81" s="32" t="n">
         <f aca="false">IF(C81="",H80,H80-G81)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I81" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I81" s="34"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="28" t="str">
         <f aca="false">IF(C82="","",MAX($B$6:B81)+1)</f>
         <v/>
       </c>
-      <c r="C82" s="34"/>
+      <c r="C82" s="35"/>
       <c r="D82" s="30"/>
       <c r="E82" s="31"/>
       <c r="F82" s="30" t="str">
@@ -3139,16 +3150,16 @@
       </c>
       <c r="H82" s="32" t="n">
         <f aca="false">IF(C82="",H81,H81-G82)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I82" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I82" s="34"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B83" s="28" t="str">
         <f aca="false">IF(C83="","",MAX($B$6:B82)+1)</f>
         <v/>
       </c>
-      <c r="C83" s="34"/>
+      <c r="C83" s="35"/>
       <c r="D83" s="30"/>
       <c r="E83" s="31"/>
       <c r="F83" s="30" t="str">
@@ -3161,16 +3172,16 @@
       </c>
       <c r="H83" s="32" t="n">
         <f aca="false">IF(C83="",H82,H82-G83)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I83" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I83" s="34"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="28" t="str">
         <f aca="false">IF(C84="","",MAX($B$6:B83)+1)</f>
         <v/>
       </c>
-      <c r="C84" s="34"/>
+      <c r="C84" s="35"/>
       <c r="D84" s="30"/>
       <c r="E84" s="31"/>
       <c r="F84" s="30" t="str">
@@ -3183,16 +3194,16 @@
       </c>
       <c r="H84" s="32" t="n">
         <f aca="false">IF(C84="",H83,H83-G84)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I84" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I84" s="34"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="28" t="str">
         <f aca="false">IF(C85="","",MAX($B$6:B84)+1)</f>
         <v/>
       </c>
-      <c r="C85" s="34"/>
+      <c r="C85" s="35"/>
       <c r="D85" s="30"/>
       <c r="E85" s="31"/>
       <c r="F85" s="30" t="str">
@@ -3205,16 +3216,16 @@
       </c>
       <c r="H85" s="32" t="n">
         <f aca="false">IF(C85="",H84,H84-G85)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I85" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I85" s="34"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B86" s="28" t="str">
         <f aca="false">IF(C86="","",MAX($B$6:B85)+1)</f>
         <v/>
       </c>
-      <c r="C86" s="34"/>
+      <c r="C86" s="35"/>
       <c r="D86" s="30"/>
       <c r="E86" s="31"/>
       <c r="F86" s="30" t="str">
@@ -3227,16 +3238,16 @@
       </c>
       <c r="H86" s="32" t="n">
         <f aca="false">IF(C86="",H85,H85-G86)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I86" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I86" s="34"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="28" t="str">
         <f aca="false">IF(C87="","",MAX($B$6:B86)+1)</f>
         <v/>
       </c>
-      <c r="C87" s="34"/>
+      <c r="C87" s="35"/>
       <c r="D87" s="30"/>
       <c r="E87" s="31"/>
       <c r="F87" s="30" t="str">
@@ -3249,16 +3260,16 @@
       </c>
       <c r="H87" s="32" t="n">
         <f aca="false">IF(C87="",H86,H86-G87)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I87" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I87" s="34"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="28" t="str">
         <f aca="false">IF(C88="","",MAX($B$6:B87)+1)</f>
         <v/>
       </c>
-      <c r="C88" s="34"/>
+      <c r="C88" s="35"/>
       <c r="D88" s="30"/>
       <c r="E88" s="31"/>
       <c r="F88" s="30" t="str">
@@ -3271,16 +3282,16 @@
       </c>
       <c r="H88" s="32" t="n">
         <f aca="false">IF(C88="",H87,H87-G88)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I88" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I88" s="34"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="28" t="str">
         <f aca="false">IF(C89="","",MAX($B$6:B88)+1)</f>
         <v/>
       </c>
-      <c r="C89" s="34"/>
+      <c r="C89" s="35"/>
       <c r="D89" s="30"/>
       <c r="E89" s="31"/>
       <c r="F89" s="30" t="str">
@@ -3293,16 +3304,16 @@
       </c>
       <c r="H89" s="32" t="n">
         <f aca="false">IF(C89="",H88,H88-G89)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I89" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I89" s="34"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B90" s="28" t="str">
         <f aca="false">IF(C90="","",MAX($B$6:B89)+1)</f>
         <v/>
       </c>
-      <c r="C90" s="34"/>
+      <c r="C90" s="35"/>
       <c r="D90" s="30"/>
       <c r="E90" s="31"/>
       <c r="F90" s="30" t="str">
@@ -3315,16 +3326,16 @@
       </c>
       <c r="H90" s="32" t="n">
         <f aca="false">IF(C90="",H89,H89-G90)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I90" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I90" s="34"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B91" s="28" t="str">
         <f aca="false">IF(C91="","",MAX($B$6:B90)+1)</f>
         <v/>
       </c>
-      <c r="C91" s="34"/>
+      <c r="C91" s="35"/>
       <c r="D91" s="30"/>
       <c r="E91" s="31"/>
       <c r="F91" s="30" t="str">
@@ -3337,16 +3348,16 @@
       </c>
       <c r="H91" s="32" t="n">
         <f aca="false">IF(C91="",H90,H90-G91)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I91" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I91" s="34"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="28" t="str">
         <f aca="false">IF(C92="","",MAX($B$6:B91)+1)</f>
         <v/>
       </c>
-      <c r="C92" s="34"/>
+      <c r="C92" s="35"/>
       <c r="D92" s="30"/>
       <c r="E92" s="31"/>
       <c r="F92" s="30" t="str">
@@ -3359,16 +3370,16 @@
       </c>
       <c r="H92" s="32" t="n">
         <f aca="false">IF(C92="",H91,H91-G92)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I92" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I92" s="34"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="28" t="str">
         <f aca="false">IF(C93="","",MAX($B$6:B92)+1)</f>
         <v/>
       </c>
-      <c r="C93" s="34"/>
+      <c r="C93" s="35"/>
       <c r="D93" s="30"/>
       <c r="E93" s="31"/>
       <c r="F93" s="30" t="str">
@@ -3381,16 +3392,16 @@
       </c>
       <c r="H93" s="32" t="n">
         <f aca="false">IF(C93="",H92,H92-G93)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I93" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I93" s="34"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="28" t="str">
         <f aca="false">IF(C94="","",MAX($B$6:B93)+1)</f>
         <v/>
       </c>
-      <c r="C94" s="34"/>
+      <c r="C94" s="35"/>
       <c r="D94" s="30"/>
       <c r="E94" s="31"/>
       <c r="F94" s="30" t="str">
@@ -3403,16 +3414,16 @@
       </c>
       <c r="H94" s="32" t="n">
         <f aca="false">IF(C94="",H93,H93-G94)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I94" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I94" s="34"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B95" s="28" t="str">
         <f aca="false">IF(C95="","",MAX($B$6:B94)+1)</f>
         <v/>
       </c>
-      <c r="C95" s="34"/>
+      <c r="C95" s="35"/>
       <c r="D95" s="30"/>
       <c r="E95" s="31"/>
       <c r="F95" s="30" t="str">
@@ -3425,16 +3436,16 @@
       </c>
       <c r="H95" s="32" t="n">
         <f aca="false">IF(C95="",H94,H94-G95)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I95" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I95" s="34"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B96" s="28" t="str">
         <f aca="false">IF(C96="","",MAX($B$6:B95)+1)</f>
         <v/>
       </c>
-      <c r="C96" s="34"/>
+      <c r="C96" s="35"/>
       <c r="D96" s="30"/>
       <c r="E96" s="31"/>
       <c r="F96" s="30" t="str">
@@ -3447,16 +3458,16 @@
       </c>
       <c r="H96" s="32" t="n">
         <f aca="false">IF(C96="",H95,H95-G96)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I96" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I96" s="34"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B97" s="28" t="str">
         <f aca="false">IF(C97="","",MAX($B$6:B96)+1)</f>
         <v/>
       </c>
-      <c r="C97" s="34"/>
+      <c r="C97" s="35"/>
       <c r="D97" s="30"/>
       <c r="E97" s="31"/>
       <c r="F97" s="30" t="str">
@@ -3469,16 +3480,16 @@
       </c>
       <c r="H97" s="32" t="n">
         <f aca="false">IF(C97="",H96,H96-G97)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I97" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I97" s="34"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B98" s="28" t="str">
         <f aca="false">IF(C98="","",MAX($B$6:B97)+1)</f>
         <v/>
       </c>
-      <c r="C98" s="34"/>
+      <c r="C98" s="35"/>
       <c r="D98" s="30"/>
       <c r="E98" s="31"/>
       <c r="F98" s="30" t="str">
@@ -3491,16 +3502,16 @@
       </c>
       <c r="H98" s="32" t="n">
         <f aca="false">IF(C98="",H97,H97-G98)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I98" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I98" s="34"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B99" s="28" t="str">
         <f aca="false">IF(C99="","",MAX($B$6:B98)+1)</f>
         <v/>
       </c>
-      <c r="C99" s="34"/>
+      <c r="C99" s="35"/>
       <c r="D99" s="30"/>
       <c r="E99" s="31"/>
       <c r="F99" s="30" t="str">
@@ -3513,16 +3524,16 @@
       </c>
       <c r="H99" s="32" t="n">
         <f aca="false">IF(C99="",H98,H98-G99)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I99" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I99" s="34"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B100" s="28" t="str">
         <f aca="false">IF(C100="","",MAX($B$6:B99)+1)</f>
         <v/>
       </c>
-      <c r="C100" s="34"/>
+      <c r="C100" s="35"/>
       <c r="D100" s="30"/>
       <c r="E100" s="31"/>
       <c r="F100" s="30" t="str">
@@ -3535,9 +3546,9 @@
       </c>
       <c r="H100" s="32" t="n">
         <f aca="false">IF(C100="",H99,H99-G100)</f>
-        <v>43356.76</v>
-      </c>
-      <c r="I100" s="35"/>
+        <v>42830.71</v>
+      </c>
+      <c r="I100" s="34"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="1" t="str">
@@ -3554,7 +3565,7 @@
       </c>
       <c r="H101" s="36" t="n">
         <f aca="false">IF(C101="",H100,H100-G101)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3572,7 +3583,7 @@
       </c>
       <c r="H102" s="36" t="n">
         <f aca="false">IF(C102="",H101,H101-G102)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3590,7 +3601,7 @@
       </c>
       <c r="H103" s="36" t="n">
         <f aca="false">IF(C103="",H102,H102-G103)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3608,7 +3619,7 @@
       </c>
       <c r="H104" s="36" t="n">
         <f aca="false">IF(C104="",H103,H103-G104)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3626,7 +3637,7 @@
       </c>
       <c r="H105" s="36" t="n">
         <f aca="false">IF(C105="",H104,H104-G105)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3644,7 +3655,7 @@
       </c>
       <c r="H106" s="36" t="n">
         <f aca="false">IF(C106="",H105,H105-G106)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3662,7 +3673,7 @@
       </c>
       <c r="H107" s="36" t="n">
         <f aca="false">IF(C107="",H106,H106-G107)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3680,7 +3691,7 @@
       </c>
       <c r="H108" s="36" t="n">
         <f aca="false">IF(C108="",H107,H107-G108)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3698,7 +3709,7 @@
       </c>
       <c r="H109" s="36" t="n">
         <f aca="false">IF(C109="",H108,H108-G109)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3716,7 +3727,7 @@
       </c>
       <c r="H110" s="36" t="n">
         <f aca="false">IF(C110="",H109,H109-G110)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3734,7 +3745,7 @@
       </c>
       <c r="H111" s="36" t="n">
         <f aca="false">IF(C111="",H110,H110-G111)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3752,7 +3763,7 @@
       </c>
       <c r="H112" s="36" t="n">
         <f aca="false">IF(C112="",H111,H111-G112)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3770,7 +3781,7 @@
       </c>
       <c r="H113" s="36" t="n">
         <f aca="false">IF(C113="",H112,H112-G113)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3788,7 +3799,7 @@
       </c>
       <c r="H114" s="36" t="n">
         <f aca="false">IF(C114="",H113,H113-G114)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3806,7 +3817,7 @@
       </c>
       <c r="H115" s="36" t="n">
         <f aca="false">IF(C115="",H114,H114-G115)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3824,7 +3835,7 @@
       </c>
       <c r="H116" s="36" t="n">
         <f aca="false">IF(C116="",H115,H115-G116)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3842,7 +3853,7 @@
       </c>
       <c r="H117" s="36" t="n">
         <f aca="false">IF(C117="",H116,H116-G117)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3860,7 +3871,7 @@
       </c>
       <c r="H118" s="36" t="n">
         <f aca="false">IF(C118="",H117,H117-G118)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3878,7 +3889,7 @@
       </c>
       <c r="H119" s="36" t="n">
         <f aca="false">IF(C119="",H118,H118-G119)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3896,7 +3907,7 @@
       </c>
       <c r="H120" s="36" t="n">
         <f aca="false">IF(C120="",H119,H119-G120)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3914,7 +3925,7 @@
       </c>
       <c r="H121" s="36" t="n">
         <f aca="false">IF(C121="",H120,H120-G121)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3932,7 +3943,7 @@
       </c>
       <c r="H122" s="36" t="n">
         <f aca="false">IF(C122="",H121,H121-G122)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3950,7 +3961,7 @@
       </c>
       <c r="H123" s="36" t="n">
         <f aca="false">IF(C123="",H122,H122-G123)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3968,7 +3979,7 @@
       </c>
       <c r="H124" s="36" t="n">
         <f aca="false">IF(C124="",H123,H123-G124)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3986,7 +3997,7 @@
       </c>
       <c r="H125" s="36" t="n">
         <f aca="false">IF(C125="",H124,H124-G125)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4004,7 +4015,7 @@
       </c>
       <c r="H126" s="36" t="n">
         <f aca="false">IF(C126="",H125,H125-G126)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4022,7 +4033,7 @@
       </c>
       <c r="H127" s="36" t="n">
         <f aca="false">IF(C127="",H126,H126-G127)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4040,7 +4051,7 @@
       </c>
       <c r="H128" s="36" t="n">
         <f aca="false">IF(C128="",H127,H127-G128)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4058,7 +4069,7 @@
       </c>
       <c r="H129" s="36" t="n">
         <f aca="false">IF(C129="",H128,H128-G129)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4076,7 +4087,7 @@
       </c>
       <c r="H130" s="36" t="n">
         <f aca="false">IF(C130="",H129,H129-G130)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4094,7 +4105,7 @@
       </c>
       <c r="H131" s="36" t="n">
         <f aca="false">IF(C131="",H130,H130-G131)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4112,7 +4123,7 @@
       </c>
       <c r="H132" s="36" t="n">
         <f aca="false">IF(C132="",H131,H131-G132)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4130,7 +4141,7 @@
       </c>
       <c r="H133" s="36" t="n">
         <f aca="false">IF(C133="",H132,H132-G133)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4148,7 +4159,7 @@
       </c>
       <c r="H134" s="36" t="n">
         <f aca="false">IF(C134="",H133,H133-G134)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4166,7 +4177,7 @@
       </c>
       <c r="H135" s="36" t="n">
         <f aca="false">IF(C135="",H134,H134-G135)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4184,7 +4195,7 @@
       </c>
       <c r="H136" s="36" t="n">
         <f aca="false">IF(C136="",H135,H135-G136)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4202,7 +4213,7 @@
       </c>
       <c r="H137" s="36" t="n">
         <f aca="false">IF(C137="",H136,H136-G137)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4220,7 +4231,7 @@
       </c>
       <c r="H138" s="36" t="n">
         <f aca="false">IF(C138="",H137,H137-G138)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4238,7 +4249,7 @@
       </c>
       <c r="H139" s="36" t="n">
         <f aca="false">IF(C139="",H138,H138-G139)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4256,7 +4267,7 @@
       </c>
       <c r="H140" s="36" t="n">
         <f aca="false">IF(C140="",H139,H139-G140)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4274,7 +4285,7 @@
       </c>
       <c r="H141" s="36" t="n">
         <f aca="false">IF(C141="",H140,H140-G141)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4292,7 +4303,7 @@
       </c>
       <c r="H142" s="36" t="n">
         <f aca="false">IF(C142="",H141,H141-G142)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4310,7 +4321,7 @@
       </c>
       <c r="H143" s="36" t="n">
         <f aca="false">IF(C143="",H142,H142-G143)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4328,7 +4339,7 @@
       </c>
       <c r="H144" s="36" t="n">
         <f aca="false">IF(C144="",H143,H143-G144)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4346,7 +4357,7 @@
       </c>
       <c r="H145" s="36" t="n">
         <f aca="false">IF(C145="",H144,H144-G145)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4364,7 +4375,7 @@
       </c>
       <c r="H146" s="36" t="n">
         <f aca="false">IF(C146="",H145,H145-G146)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4382,7 +4393,7 @@
       </c>
       <c r="H147" s="36" t="n">
         <f aca="false">IF(C147="",H146,H146-G147)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4400,7 +4411,7 @@
       </c>
       <c r="H148" s="36" t="n">
         <f aca="false">IF(C148="",H147,H147-G148)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4418,7 +4429,7 @@
       </c>
       <c r="H149" s="36" t="n">
         <f aca="false">IF(C149="",H148,H148-G149)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4436,7 +4447,7 @@
       </c>
       <c r="H150" s="36" t="n">
         <f aca="false">IF(C150="",H149,H149-G150)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4454,7 +4465,7 @@
       </c>
       <c r="H151" s="36" t="n">
         <f aca="false">IF(C151="",H150,H150-G151)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4472,7 +4483,7 @@
       </c>
       <c r="H152" s="36" t="n">
         <f aca="false">IF(C152="",H151,H151-G152)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4490,7 +4501,7 @@
       </c>
       <c r="H153" s="36" t="n">
         <f aca="false">IF(C153="",H152,H152-G153)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4508,7 +4519,7 @@
       </c>
       <c r="H154" s="36" t="n">
         <f aca="false">IF(C154="",H153,H153-G154)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4526,7 +4537,7 @@
       </c>
       <c r="H155" s="36" t="n">
         <f aca="false">IF(C155="",H154,H154-G155)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4544,7 +4555,7 @@
       </c>
       <c r="H156" s="36" t="n">
         <f aca="false">IF(C156="",H155,H155-G156)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4562,7 +4573,7 @@
       </c>
       <c r="H157" s="36" t="n">
         <f aca="false">IF(C157="",H156,H156-G157)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4580,7 +4591,7 @@
       </c>
       <c r="H158" s="36" t="n">
         <f aca="false">IF(C158="",H157,H157-G158)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4598,7 +4609,7 @@
       </c>
       <c r="H159" s="36" t="n">
         <f aca="false">IF(C159="",H158,H158-G159)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4616,7 +4627,7 @@
       </c>
       <c r="H160" s="36" t="n">
         <f aca="false">IF(C160="",H159,H159-G160)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4634,7 +4645,7 @@
       </c>
       <c r="H161" s="36" t="n">
         <f aca="false">IF(C161="",H160,H160-G161)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4652,7 +4663,7 @@
       </c>
       <c r="H162" s="36" t="n">
         <f aca="false">IF(C162="",H161,H161-G162)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4670,7 +4681,7 @@
       </c>
       <c r="H163" s="36" t="n">
         <f aca="false">IF(C163="",H162,H162-G163)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4688,7 +4699,7 @@
       </c>
       <c r="H164" s="36" t="n">
         <f aca="false">IF(C164="",H163,H163-G164)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4706,7 +4717,7 @@
       </c>
       <c r="H165" s="36" t="n">
         <f aca="false">IF(C165="",H164,H164-G165)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4724,7 +4735,7 @@
       </c>
       <c r="H166" s="36" t="n">
         <f aca="false">IF(C166="",H165,H165-G166)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4742,7 +4753,7 @@
       </c>
       <c r="H167" s="36" t="n">
         <f aca="false">IF(C167="",H166,H166-G167)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4760,7 +4771,7 @@
       </c>
       <c r="H168" s="36" t="n">
         <f aca="false">IF(C168="",H167,H167-G168)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4778,7 +4789,7 @@
       </c>
       <c r="H169" s="36" t="n">
         <f aca="false">IF(C169="",H168,H168-G169)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4796,7 +4807,7 @@
       </c>
       <c r="H170" s="36" t="n">
         <f aca="false">IF(C170="",H169,H169-G170)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4814,7 +4825,7 @@
       </c>
       <c r="H171" s="36" t="n">
         <f aca="false">IF(C171="",H170,H170-G171)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4832,7 +4843,7 @@
       </c>
       <c r="H172" s="36" t="n">
         <f aca="false">IF(C172="",H171,H171-G172)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4850,7 +4861,7 @@
       </c>
       <c r="H173" s="36" t="n">
         <f aca="false">IF(C173="",H172,H172-G173)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4868,7 +4879,7 @@
       </c>
       <c r="H174" s="36" t="n">
         <f aca="false">IF(C174="",H173,H173-G174)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4886,7 +4897,7 @@
       </c>
       <c r="H175" s="36" t="n">
         <f aca="false">IF(C175="",H174,H174-G175)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4904,7 +4915,7 @@
       </c>
       <c r="H176" s="36" t="n">
         <f aca="false">IF(C176="",H175,H175-G176)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4922,7 +4933,7 @@
       </c>
       <c r="H177" s="36" t="n">
         <f aca="false">IF(C177="",H176,H176-G177)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4940,7 +4951,7 @@
       </c>
       <c r="H178" s="36" t="n">
         <f aca="false">IF(C178="",H177,H177-G178)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4958,7 +4969,7 @@
       </c>
       <c r="H179" s="36" t="n">
         <f aca="false">IF(C179="",H178,H178-G179)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4976,7 +4987,7 @@
       </c>
       <c r="H180" s="36" t="n">
         <f aca="false">IF(C180="",H179,H179-G180)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4994,7 +5005,7 @@
       </c>
       <c r="H181" s="36" t="n">
         <f aca="false">IF(C181="",H180,H180-G181)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5012,7 +5023,7 @@
       </c>
       <c r="H182" s="36" t="n">
         <f aca="false">IF(C182="",H181,H181-G182)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5030,7 +5041,7 @@
       </c>
       <c r="H183" s="36" t="n">
         <f aca="false">IF(C183="",H182,H182-G183)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5048,7 +5059,7 @@
       </c>
       <c r="H184" s="36" t="n">
         <f aca="false">IF(C184="",H183,H183-G184)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5066,7 +5077,7 @@
       </c>
       <c r="H185" s="36" t="n">
         <f aca="false">IF(C185="",H184,H184-G185)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5084,7 +5095,7 @@
       </c>
       <c r="H186" s="36" t="n">
         <f aca="false">IF(C186="",H185,H185-G186)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5102,7 +5113,7 @@
       </c>
       <c r="H187" s="36" t="n">
         <f aca="false">IF(C187="",H186,H186-G187)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5120,7 +5131,7 @@
       </c>
       <c r="H188" s="36" t="n">
         <f aca="false">IF(C188="",H187,H187-G188)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5138,7 +5149,7 @@
       </c>
       <c r="H189" s="36" t="n">
         <f aca="false">IF(C189="",H188,H188-G189)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5156,7 +5167,7 @@
       </c>
       <c r="H190" s="36" t="n">
         <f aca="false">IF(C190="",H189,H189-G190)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5174,7 +5185,7 @@
       </c>
       <c r="H191" s="36" t="n">
         <f aca="false">IF(C191="",H190,H190-G191)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5192,7 +5203,7 @@
       </c>
       <c r="H192" s="36" t="n">
         <f aca="false">IF(C192="",H191,H191-G192)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5210,7 +5221,7 @@
       </c>
       <c r="H193" s="36" t="n">
         <f aca="false">IF(C193="",H192,H192-G193)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5228,7 +5239,7 @@
       </c>
       <c r="H194" s="36" t="n">
         <f aca="false">IF(C194="",H193,H193-G194)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5246,7 +5257,7 @@
       </c>
       <c r="H195" s="36" t="n">
         <f aca="false">IF(C195="",H194,H194-G195)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5264,7 +5275,7 @@
       </c>
       <c r="H196" s="36" t="n">
         <f aca="false">IF(C196="",H195,H195-G196)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5282,7 +5293,7 @@
       </c>
       <c r="H197" s="36" t="n">
         <f aca="false">IF(C197="",H196,H196-G197)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5300,7 +5311,7 @@
       </c>
       <c r="H198" s="36" t="n">
         <f aca="false">IF(C198="",H197,H197-G198)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5318,7 +5329,7 @@
       </c>
       <c r="H199" s="36" t="n">
         <f aca="false">IF(C199="",H198,H198-G199)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5336,7 +5347,7 @@
       </c>
       <c r="H200" s="36" t="n">
         <f aca="false">IF(C200="",H199,H199-G200)</f>
-        <v>43356.76</v>
+        <v>42830.71</v>
       </c>
     </row>
   </sheetData>
@@ -5395,7 +5406,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="21" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="21"/>
       <c r="D2" s="21"/>
@@ -5405,7 +5416,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -5421,7 +5432,7 @@
         <v>31</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E5" s="37" t="s">
         <v>34</v>
@@ -5437,7 +5448,7 @@
       <c r="B6" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="35" t="n">
         <v>45935</v>
       </c>
       <c r="D6" s="30" t="n">
@@ -5477,7 +5488,7 @@
       <c r="B8" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="35" t="n">
         <v>45996</v>
       </c>
       <c r="D8" s="30" t="n">
@@ -5517,7 +5528,7 @@
       <c r="B10" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="34" t="n">
+      <c r="C10" s="35" t="n">
         <v>46058</v>
       </c>
       <c r="D10" s="30" t="n">
@@ -5557,7 +5568,7 @@
       <c r="B12" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="34" t="n">
+      <c r="C12" s="35" t="n">
         <v>46117</v>
       </c>
       <c r="D12" s="30" t="n">
@@ -5597,7 +5608,7 @@
       <c r="B14" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="C14" s="34" t="n">
+      <c r="C14" s="35" t="n">
         <v>46178</v>
       </c>
       <c r="D14" s="30" t="n">
@@ -5637,7 +5648,7 @@
       <c r="B16" s="31" t="n">
         <v>11</v>
       </c>
-      <c r="C16" s="34" t="n">
+      <c r="C16" s="35" t="n">
         <v>46239</v>
       </c>
       <c r="D16" s="30" t="n">
@@ -5677,7 +5688,7 @@
       <c r="B18" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="C18" s="34" t="n">
+      <c r="C18" s="35" t="n">
         <v>46300</v>
       </c>
       <c r="D18" s="30" t="n">
@@ -5717,7 +5728,7 @@
       <c r="B20" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="34" t="n">
+      <c r="C20" s="35" t="n">
         <v>46361</v>
       </c>
       <c r="D20" s="30" t="n">
@@ -5757,7 +5768,7 @@
       <c r="B22" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="C22" s="34" t="n">
+      <c r="C22" s="35" t="n">
         <v>46423</v>
       </c>
       <c r="D22" s="30" t="n">
@@ -5797,7 +5808,7 @@
       <c r="B24" s="31" t="n">
         <v>19</v>
       </c>
-      <c r="C24" s="34" t="n">
+      <c r="C24" s="35" t="n">
         <v>46482</v>
       </c>
       <c r="D24" s="30" t="n">
@@ -5837,7 +5848,7 @@
       <c r="B26" s="31" t="n">
         <v>21</v>
       </c>
-      <c r="C26" s="34" t="n">
+      <c r="C26" s="35" t="n">
         <v>46543</v>
       </c>
       <c r="D26" s="30" t="n">
@@ -5877,7 +5888,7 @@
       <c r="B28" s="31" t="n">
         <v>23</v>
       </c>
-      <c r="C28" s="34" t="n">
+      <c r="C28" s="35" t="n">
         <v>46604</v>
       </c>
       <c r="D28" s="30" t="n">
@@ -5917,7 +5928,7 @@
       <c r="B30" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="C30" s="34" t="n">
+      <c r="C30" s="35" t="n">
         <v>46665</v>
       </c>
       <c r="D30" s="30" t="n">
@@ -5957,7 +5968,7 @@
       <c r="B32" s="31" t="n">
         <v>27</v>
       </c>
-      <c r="C32" s="34" t="n">
+      <c r="C32" s="35" t="n">
         <v>46726</v>
       </c>
       <c r="D32" s="30" t="n">
@@ -5997,7 +6008,7 @@
       <c r="B34" s="31" t="n">
         <v>29</v>
       </c>
-      <c r="C34" s="34" t="n">
+      <c r="C34" s="35" t="n">
         <v>46788</v>
       </c>
       <c r="D34" s="30" t="n">
@@ -6037,7 +6048,7 @@
       <c r="B36" s="31" t="n">
         <v>31</v>
       </c>
-      <c r="C36" s="34" t="n">
+      <c r="C36" s="35" t="n">
         <v>46848</v>
       </c>
       <c r="D36" s="30" t="n">
@@ -6077,7 +6088,7 @@
       <c r="B38" s="31" t="n">
         <v>33</v>
       </c>
-      <c r="C38" s="34" t="n">
+      <c r="C38" s="35" t="n">
         <v>46909</v>
       </c>
       <c r="D38" s="30" t="n">
@@ -6117,7 +6128,7 @@
       <c r="B40" s="31" t="n">
         <v>35</v>
       </c>
-      <c r="C40" s="34" t="n">
+      <c r="C40" s="35" t="n">
         <v>46970</v>
       </c>
       <c r="D40" s="30" t="n">
@@ -6157,7 +6168,7 @@
       <c r="B42" s="31" t="n">
         <v>37</v>
       </c>
-      <c r="C42" s="34" t="n">
+      <c r="C42" s="35" t="n">
         <v>47031</v>
       </c>
       <c r="D42" s="30" t="n">
@@ -6197,7 +6208,7 @@
       <c r="B44" s="31" t="n">
         <v>39</v>
       </c>
-      <c r="C44" s="34" t="n">
+      <c r="C44" s="35" t="n">
         <v>47092</v>
       </c>
       <c r="D44" s="30" t="n">
@@ -6237,7 +6248,7 @@
       <c r="B46" s="31" t="n">
         <v>41</v>
       </c>
-      <c r="C46" s="34" t="n">
+      <c r="C46" s="35" t="n">
         <v>47154</v>
       </c>
       <c r="D46" s="30" t="n">
@@ -6277,7 +6288,7 @@
       <c r="B48" s="31" t="n">
         <v>43</v>
       </c>
-      <c r="C48" s="34" t="n">
+      <c r="C48" s="35" t="n">
         <v>47213</v>
       </c>
       <c r="D48" s="30" t="n">
@@ -6317,7 +6328,7 @@
       <c r="B50" s="31" t="n">
         <v>45</v>
       </c>
-      <c r="C50" s="34" t="n">
+      <c r="C50" s="35" t="n">
         <v>47274</v>
       </c>
       <c r="D50" s="30" t="n">
@@ -6357,7 +6368,7 @@
       <c r="B52" s="31" t="n">
         <v>47</v>
       </c>
-      <c r="C52" s="34" t="n">
+      <c r="C52" s="35" t="n">
         <v>47335</v>
       </c>
       <c r="D52" s="30" t="n">
@@ -6397,7 +6408,7 @@
       <c r="B54" s="31" t="n">
         <v>49</v>
       </c>
-      <c r="C54" s="34" t="n">
+      <c r="C54" s="35" t="n">
         <v>47396</v>
       </c>
       <c r="D54" s="30" t="n">
@@ -6437,7 +6448,7 @@
       <c r="B56" s="31" t="n">
         <v>51</v>
       </c>
-      <c r="C56" s="34" t="n">
+      <c r="C56" s="35" t="n">
         <v>47457</v>
       </c>
       <c r="D56" s="30" t="n">
@@ -6477,7 +6488,7 @@
       <c r="B58" s="31" t="n">
         <v>53</v>
       </c>
-      <c r="C58" s="34" t="n">
+      <c r="C58" s="35" t="n">
         <v>47519</v>
       </c>
       <c r="D58" s="30" t="n">
@@ -6517,7 +6528,7 @@
       <c r="B60" s="31" t="n">
         <v>55</v>
       </c>
-      <c r="C60" s="34" t="n">
+      <c r="C60" s="35" t="n">
         <v>47578</v>
       </c>
       <c r="D60" s="30" t="n">
@@ -6557,7 +6568,7 @@
       <c r="B62" s="31" t="n">
         <v>57</v>
       </c>
-      <c r="C62" s="34" t="n">
+      <c r="C62" s="35" t="n">
         <v>47639</v>
       </c>
       <c r="D62" s="30" t="n">
@@ -6597,7 +6608,7 @@
       <c r="B64" s="31" t="n">
         <v>59</v>
       </c>
-      <c r="C64" s="34" t="n">
+      <c r="C64" s="35" t="n">
         <v>47700</v>
       </c>
       <c r="D64" s="30" t="n">
@@ -6637,7 +6648,7 @@
       <c r="B66" s="31" t="n">
         <v>61</v>
       </c>
-      <c r="C66" s="34" t="n">
+      <c r="C66" s="35" t="n">
         <v>47761</v>
       </c>
       <c r="D66" s="30" t="n">
@@ -6677,7 +6688,7 @@
       <c r="B68" s="31" t="n">
         <v>63</v>
       </c>
-      <c r="C68" s="34" t="n">
+      <c r="C68" s="35" t="n">
         <v>47822</v>
       </c>
       <c r="D68" s="30" t="n">
@@ -6717,7 +6728,7 @@
       <c r="B70" s="31" t="n">
         <v>65</v>
       </c>
-      <c r="C70" s="34" t="n">
+      <c r="C70" s="35" t="n">
         <v>47884</v>
       </c>
       <c r="D70" s="30" t="n">
@@ -6757,7 +6768,7 @@
       <c r="B72" s="31" t="n">
         <v>67</v>
       </c>
-      <c r="C72" s="34" t="n">
+      <c r="C72" s="35" t="n">
         <v>47943</v>
       </c>
       <c r="D72" s="30" t="n">
@@ -6797,7 +6808,7 @@
       <c r="B74" s="31" t="n">
         <v>69</v>
       </c>
-      <c r="C74" s="34" t="n">
+      <c r="C74" s="35" t="n">
         <v>48004</v>
       </c>
       <c r="D74" s="30" t="n">
@@ -6837,7 +6848,7 @@
       <c r="B76" s="31" t="n">
         <v>71</v>
       </c>
-      <c r="C76" s="34" t="n">
+      <c r="C76" s="35" t="n">
         <v>48065</v>
       </c>
       <c r="D76" s="30" t="n">
@@ -6877,7 +6888,7 @@
       <c r="B78" s="31" t="n">
         <v>73</v>
       </c>
-      <c r="C78" s="34" t="n">
+      <c r="C78" s="35" t="n">
         <v>48126</v>
       </c>
       <c r="D78" s="30" t="n">
@@ -6917,7 +6928,7 @@
       <c r="B80" s="31" t="n">
         <v>75</v>
       </c>
-      <c r="C80" s="34" t="n">
+      <c r="C80" s="35" t="n">
         <v>48187</v>
       </c>
       <c r="D80" s="30" t="n">
@@ -6957,7 +6968,7 @@
       <c r="B82" s="31" t="n">
         <v>77</v>
       </c>
-      <c r="C82" s="34" t="n">
+      <c r="C82" s="35" t="n">
         <v>48249</v>
       </c>
       <c r="D82" s="30" t="n">
@@ -6997,7 +7008,7 @@
       <c r="B84" s="31" t="n">
         <v>79</v>
       </c>
-      <c r="C84" s="34" t="n">
+      <c r="C84" s="35" t="n">
         <v>48309</v>
       </c>
       <c r="D84" s="30" t="n">
@@ -7037,7 +7048,7 @@
       <c r="B86" s="31" t="n">
         <v>81</v>
       </c>
-      <c r="C86" s="34" t="n">
+      <c r="C86" s="35" t="n">
         <v>48370</v>
       </c>
       <c r="D86" s="30" t="n">
@@ -7077,7 +7088,7 @@
       <c r="B88" s="31" t="n">
         <v>83</v>
       </c>
-      <c r="C88" s="34" t="n">
+      <c r="C88" s="35" t="n">
         <v>48431</v>
       </c>
       <c r="D88" s="30" t="n">

</xml_diff>

<commit_message>
Marcela payoff quote correction — accrual from Jul 1 (16 days), $42,924.59
</commit_message>
<xml_diff>
--- a/public/marcela/Marcela_Loan_Tracker.xlsx
+++ b/public/marcela/Marcela_Loan_Tracker.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -136,13 +136,13 @@
     <t xml:space="preserve">Total Payoff Amount</t>
   </si>
   <si>
-    <t xml:space="preserve">Days Since Last Payment</t>
+    <t xml:space="preserve">Days Accrued This Month</t>
   </si>
   <si>
     <t xml:space="preserve">Interest Saved vs. Maturity</t>
   </si>
   <si>
-    <t xml:space="preserve">Method. 5.00% APR fixed, actual/365 daily accrual on outstanding principal from the last payment date to the payoff date. No prepayment penalty. Payoff quote issued 7/14/2026; letter delivered same day.</t>
+    <t xml:space="preserve">Method. 5.00% APR fixed, actual/365 daily accrual on outstanding principal from the first day of the payoff month to the payoff date. No prepayment penalty. Payoff quote reissued 7/16/2026; letter updated same day.</t>
   </si>
   <si>
     <t xml:space="preserve">Payment Register</t>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="F33" s="24" t="n">
         <f aca="false">IF(C35="","",ROUND(C34*C7/365*C35,2))</f>
-        <v>105.61</v>
+        <v>93.88</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="F34" s="25" t="n">
         <f aca="false">IF(F33="","",C34+F33)</f>
-        <v>42936.32</v>
+        <v>42924.59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1336,8 +1336,8 @@
         <v>36</v>
       </c>
       <c r="C35" s="26" t="n">
-        <f aca="false">IF(OR(C32="",C33=""),"",C32-C33)</f>
-        <v>18</v>
+        <f aca="false">IF(OR(C32="",C33=""),"",C32-DATE(YEAR(C32),MONTH(C32),1))</f>
+        <v>16</v>
       </c>
       <c r="D35" s="18"/>
       <c r="E35" s="6" t="s">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F35" s="24" t="n">
         <f aca="false">IF(F34="","",ROUND(F7*C12-F34,2))</f>
-        <v>6532.68</v>
+        <v>6544.41</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Marcela payoff correction — pmt #14 satisfied Jul 5, payoff = $42,830.71 flat
</commit_message>
<xml_diff>
--- a/public/marcela/Marcela_Loan_Tracker.xlsx
+++ b/public/marcela/Marcela_Loan_Tracker.xlsx
@@ -124,7 +124,7 @@
     <t xml:space="preserve">Per Diem Interest</t>
   </si>
   <si>
-    <t xml:space="preserve">Last Payment Date</t>
+    <t xml:space="preserve">Next Scheduled Due Date</t>
   </si>
   <si>
     <t xml:space="preserve">Accrued Interest (Actual/365)</t>
@@ -136,13 +136,13 @@
     <t xml:space="preserve">Total Payoff Amount</t>
   </si>
   <si>
-    <t xml:space="preserve">Days Accrued This Month</t>
+    <t xml:space="preserve">Days Accrued Since Due Date</t>
   </si>
   <si>
     <t xml:space="preserve">Interest Saved vs. Maturity</t>
   </si>
   <si>
-    <t xml:space="preserve">Method. 5.00% APR fixed, actual/365 daily accrual on outstanding principal from the first day of the payoff month to the payoff date. No prepayment penalty. Payoff quote reissued 7/16/2026; letter updated same day.</t>
+    <t xml:space="preserve">Method. 5.00% APR fixed, actual/365 daily accrual on outstanding principal. Payment #14 (received 6/29/2026, memo "Pool loan payment July 1 2026") satisfied the July 5, 2026 installment early, so no interest accrues for a payoff on or before the next scheduled due date of August 5, 2026. No prepayment penalty. Payoff quote reissued 7/16/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Payment Register</t>
@@ -1302,8 +1302,8 @@
         <v>32</v>
       </c>
       <c r="C33" s="23" t="n">
-        <f aca="false">LOOKUP(2,1/('Payment Register'!D7:D200&lt;&gt;""),'Payment Register'!C7:C200)</f>
-        <v>46202</v>
+        <f aca="false">DATE(2026,8,5)</f>
+        <v>46239</v>
       </c>
       <c r="D33" s="18"/>
       <c r="E33" s="6" t="s">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="F33" s="24" t="n">
         <f aca="false">IF(C35="","",ROUND(C34*C7/365*C35,2))</f>
-        <v>93.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="F34" s="25" t="n">
         <f aca="false">IF(F33="","",C34+F33)</f>
-        <v>42924.59</v>
+        <v>42830.71</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1336,8 +1336,8 @@
         <v>36</v>
       </c>
       <c r="C35" s="26" t="n">
-        <f aca="false">IF(OR(C32="",C33=""),"",C32-DATE(YEAR(C32),MONTH(C32),1))</f>
-        <v>16</v>
+        <f aca="false">IF(OR(C32="",C33=""),"",MAX(0,C32-C33))</f>
+        <v>0</v>
       </c>
       <c r="D35" s="18"/>
       <c r="E35" s="6" t="s">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F35" s="24" t="n">
         <f aca="false">IF(F34="","",ROUND(F7*C12-F34,2))</f>
-        <v>6544.41</v>
+        <v>6638.29</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>